<commit_message>
Day 36 Folder added Polymorphism Revision
</commit_message>
<xml_diff>
--- a/Java Full Stack.xlsx
+++ b/Java Full Stack.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Kodewala Academy\Java Full Stack Backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Kodewala Academy\Java Full Stack (Backend)\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05CB0544-FDA9-488A-BB0B-C4080EB9B5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1166B4D9-B9DA-4DB3-9A2F-71B8309E97E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="116">
   <si>
     <t>Date</t>
   </si>
@@ -368,6 +368,24 @@
   </si>
   <si>
     <t>Polymorphism- Auto Up scaling and down scaling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://us06web.zoom.us/rec/share/IwBzpR0D-FcNFDW8fUJLY44n3gksyic0vVHBg8YEqX5Or4N81YNGh4VeRD15U2A4.Y5ITMz0BcphZcT-- </t>
+  </si>
+  <si>
+    <t>Passcode: aer1k=eg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://us06web.zoom.us/rec/share/V1boQRNCoIgxz6w2djpHHgDx9JuIxtdoqt2YYkSO8ZUysHb0-zLpwZMKEO6e_Z0X.J_zcc1PXunhW135K </t>
+  </si>
+  <si>
+    <t>Passcode: 7!j$6yi+</t>
+  </si>
+  <si>
+    <t>Revision- Inheritance, Encapsulation, Abstraction and Override</t>
+  </si>
+  <si>
+    <t>Revision - Polymorphism</t>
   </si>
 </sst>
 </file>
@@ -513,7 +531,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -549,9 +567,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -840,7 +855,7 @@
   <cols>
     <col min="1" max="1" width="6.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.28515625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="57" style="1" customWidth="1"/>
+    <col min="3" max="3" width="61.85546875" style="1" customWidth="1"/>
     <col min="4" max="4" width="129" style="1" customWidth="1"/>
     <col min="5" max="5" width="22.28515625" style="1" customWidth="1"/>
     <col min="6" max="16384" width="9.140625" style="1"/>
@@ -1478,25 +1493,43 @@
       <c r="A39" s="2">
         <v>35</v>
       </c>
-      <c r="B39" s="2"/>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
+      <c r="B39" s="5">
+        <v>46321</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>36</v>
       </c>
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
+      <c r="B40" s="5">
+        <v>46322</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2">
         <v>37</v>
       </c>
-      <c r="B41" s="2"/>
+      <c r="B41" s="5">
+        <v>46323</v>
+      </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -1505,7 +1538,9 @@
       <c r="A42" s="2">
         <v>38</v>
       </c>
-      <c r="B42" s="2"/>
+      <c r="B42" s="5">
+        <v>46324</v>
+      </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -1514,9 +1549,12 @@
       <c r="A43" s="2">
         <v>39</v>
       </c>
-      <c r="B43" s="2"/>
+      <c r="B43" s="5">
+        <v>46325</v>
+      </c>
       <c r="C43" s="2"/>
-      <c r="E43" s="13"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2">

</xml_diff>